<commit_message>
Drop the owl emoji from menu, sheet and page names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kPBSYq9ZY5XtdXkATthy6
</commit_message>
<xml_diff>
--- a/sova-report/sova-report.xlsx
+++ b/sova-report/sova-report.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="🦉 Сводная" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Сводная" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Направление 1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Направление 2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Направление 3" sheetId="4" state="visible" r:id="rId4"/>
@@ -459,7 +459,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'🦉 Сводная'!E19</f>
+              <f>'Сводная'!E19</f>
             </strRef>
           </tx>
           <spPr>
@@ -488,12 +488,12 @@
           </trendline>
           <cat>
             <numRef>
-              <f>'🦉 Сводная'!$A$20:$A$45</f>
+              <f>'Сводная'!$A$20:$A$45</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🦉 Сводная'!$E$20:$E$45</f>
+              <f>'Сводная'!$E$20:$E$45</f>
             </numRef>
           </val>
         </ser>
@@ -654,7 +654,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'🦉 Сводная'!E106</f>
+              <f>'Сводная'!E106</f>
             </strRef>
           </tx>
           <spPr>
@@ -683,12 +683,12 @@
           </trendline>
           <cat>
             <numRef>
-              <f>'🦉 Сводная'!$A$107:$A$118</f>
+              <f>'Сводная'!$A$107:$A$118</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🦉 Сводная'!$E$107:$E$118</f>
+              <f>'Сводная'!$E$107:$E$118</f>
             </numRef>
           </val>
         </ser>
@@ -755,7 +755,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'🦉 Сводная'!B19</f>
+              <f>'Сводная'!B19</f>
             </strRef>
           </tx>
           <spPr>
@@ -776,12 +776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🦉 Сводная'!$A$20:$A$45</f>
+              <f>'Сводная'!$A$20:$A$45</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🦉 Сводная'!$B$20:$B$45</f>
+              <f>'Сводная'!$B$20:$B$45</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -791,7 +791,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'🦉 Сводная'!C19</f>
+              <f>'Сводная'!C19</f>
             </strRef>
           </tx>
           <spPr>
@@ -812,12 +812,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🦉 Сводная'!$A$20:$A$45</f>
+              <f>'Сводная'!$A$20:$A$45</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🦉 Сводная'!$C$20:$C$45</f>
+              <f>'Сводная'!$C$20:$C$45</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -827,7 +827,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'🦉 Сводная'!D19</f>
+              <f>'Сводная'!D19</f>
             </strRef>
           </tx>
           <spPr>
@@ -848,12 +848,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🦉 Сводная'!$A$20:$A$45</f>
+              <f>'Сводная'!$A$20:$A$45</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🦉 Сводная'!$D$20:$D$45</f>
+              <f>'Сводная'!$D$20:$D$45</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -923,7 +923,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'🦉 Сводная'!B106</f>
+              <f>'Сводная'!B106</f>
             </strRef>
           </tx>
           <spPr>
@@ -944,12 +944,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🦉 Сводная'!$A$107:$A$118</f>
+              <f>'Сводная'!$A$107:$A$118</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🦉 Сводная'!$B$107:$B$118</f>
+              <f>'Сводная'!$B$107:$B$118</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -959,7 +959,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'🦉 Сводная'!C106</f>
+              <f>'Сводная'!C106</f>
             </strRef>
           </tx>
           <spPr>
@@ -980,12 +980,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🦉 Сводная'!$A$107:$A$118</f>
+              <f>'Сводная'!$A$107:$A$118</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🦉 Сводная'!$C$107:$C$118</f>
+              <f>'Сводная'!$C$107:$C$118</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -995,7 +995,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'🦉 Сводная'!D106</f>
+              <f>'Сводная'!D106</f>
             </strRef>
           </tx>
           <spPr>
@@ -1016,12 +1016,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'🦉 Сводная'!$A$107:$A$118</f>
+              <f>'Сводная'!$A$107:$A$118</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'🦉 Сводная'!$D$107:$D$118</f>
+              <f>'Сводная'!$D$107:$D$118</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -2106,7 +2106,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🦉 Сова · Сводная по всем направлениям</t>
+          <t>Сова · Сводная по всем направлениям</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -5663,7 +5663,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1">
-        <f>"🦉 Сова · "&amp;$B$3</f>
+        <f>"Сова · "&amp;$B$3</f>
         <v/>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -9547,7 +9547,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1">
-        <f>"🦉 Сова · "&amp;$B$3</f>
+        <f>"Сова · "&amp;$B$3</f>
         <v/>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -13431,7 +13431,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1">
-        <f>"🦉 Сова · "&amp;$B$3</f>
+        <f>"Сова · "&amp;$B$3</f>
         <v/>
       </c>
       <c r="B1" s="2" t="n"/>

</xml_diff>

<commit_message>
Add the custom date range to every direction sheet
Each direction sheet gets its own "Период с / по" fields, working like
the summary's: the KPI block covers the chosen range and compares it
with the previous range of the same length. Each sheet keeps its range
on rebuild.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kPBSYq9ZY5XtdXkATthy6
</commit_message>
<xml_diff>
--- a/sova-report/sova-report.xlsx
+++ b/sova-report/sova-report.xlsx
@@ -75,6 +75,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="006B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F2430"/>
       <sz val="12"/>
@@ -90,11 +95,6 @@
       <b val="1"/>
       <color rgb="006B7280"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="006B7280"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -142,6 +142,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF6D6"/>
+        <bgColor rgb="00FFF6D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
@@ -150,12 +156,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F4F6FA"/>
         <bgColor rgb="00F4F6FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF6D6"/>
-        <bgColor rgb="00FFF6D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -174,11 +174,6 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="thin">
-        <color rgb="00DFE3EB"/>
-      </bottom>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="00E0C46C"/>
       </left>
@@ -190,6 +185,11 @@
       </top>
       <bottom style="thin">
         <color rgb="00E0C46C"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00DFE3EB"/>
       </bottom>
     </border>
     <border>
@@ -217,105 +217,105 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -340,28 +340,28 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="170" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -5816,17 +5816,34 @@
         <f>'⚙ Настройки'!$B$7</f>
         <v/>
       </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Период с</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>по</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="n"/>
       <c r="M3" s="9" t="inlineStr">
         <is>
           <t>📈 По дням, последние 90</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="H4" s="10">
+        <f>IF(AND(ISNUMBER(H3),ISNUMBER(J3),H3&gt;J3),"⚠ Дата «с» позже даты «по»",IF(OR(ISNUMBER(H3),ISNUMBER(J3)),"Сравнение — с предыдущим периодом той же длины. Очистите поля, чтобы вернуть текущий месяц.","Пусто — текущий месяц. Дату выбирают двойным щелчком."))</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Этот месяц против тех же дней прошлого</t>
-        </is>
+      <c r="A5" s="9">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Выбранный период против предыдущего той же длины","Этот месяц против тех же дней прошлого")</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -5887,10 +5904,9 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Этот месяц</t>
-        </is>
+      <c r="A7" s="12">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Выбранный период","Этот месяц")</f>
+        <v/>
       </c>
       <c r="B7" s="13">
         <f>SUMIFS('Данные'!$C:$C,'Данные'!$A:$A,"&gt;="&amp;$J$7,'Данные'!$A:$A,"&lt;"&amp;$K$7+1,'Данные'!$B:$B,$B$3)</f>
@@ -5925,19 +5941,18 @@
         <v/>
       </c>
       <c r="J7" s="18">
-        <f>DATE(YEAR($E$3),MONTH($E$3),1)</f>
+        <f>IF(ISNUMBER($H$3),$H$3,DATE(YEAR(K7),MONTH(K7),1))</f>
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>$E$3</f>
+        <f>IF(ISNUMBER($J$3),$J$3,$E$3)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>Прошлый, те же дни</t>
-        </is>
+      <c r="A8" s="19">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Предыдущий, той же длины","Прошлый, те же дни")</f>
+        <v/>
       </c>
       <c r="B8" s="20">
         <f>SUMIFS('Данные'!$C:$C,'Данные'!$A:$A,"&gt;="&amp;$J$8,'Данные'!$A:$A,"&lt;"&amp;$K$8+1,'Данные'!$B:$B,$B$3)</f>
@@ -5972,11 +5987,11 @@
         <v/>
       </c>
       <c r="J8" s="25">
-        <f>IF(FALSE,2*J7-K7-1,EDATE(J7,-1))</f>
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),2*J7-K7-1,EDATE(J7,-1))</f>
         <v/>
       </c>
       <c r="K8" s="25">
-        <f>IF(FALSE,J7-1,EDATE(K7,-1))</f>
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),J7-1,EDATE(K7,-1))</f>
         <v/>
       </c>
     </row>
@@ -9564,6 +9579,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H3 J3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Период" prompt="Дата. Пусто — текущий месяц." type="date" operator="greaterThan">
+      <formula1>1</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -9700,17 +9720,34 @@
         <f>'⚙ Настройки'!$B$7</f>
         <v/>
       </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Период с</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>по</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="n"/>
       <c r="M3" s="9" t="inlineStr">
         <is>
           <t>📈 По дням, последние 90</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="H4" s="10">
+        <f>IF(AND(ISNUMBER(H3),ISNUMBER(J3),H3&gt;J3),"⚠ Дата «с» позже даты «по»",IF(OR(ISNUMBER(H3),ISNUMBER(J3)),"Сравнение — с предыдущим периодом той же длины. Очистите поля, чтобы вернуть текущий месяц.","Пусто — текущий месяц. Дату выбирают двойным щелчком."))</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Этот месяц против тех же дней прошлого</t>
-        </is>
+      <c r="A5" s="9">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Выбранный период против предыдущего той же длины","Этот месяц против тех же дней прошлого")</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -9771,10 +9808,9 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Этот месяц</t>
-        </is>
+      <c r="A7" s="12">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Выбранный период","Этот месяц")</f>
+        <v/>
       </c>
       <c r="B7" s="13">
         <f>SUMIFS('Данные'!$C:$C,'Данные'!$A:$A,"&gt;="&amp;$J$7,'Данные'!$A:$A,"&lt;"&amp;$K$7+1,'Данные'!$B:$B,$B$3)</f>
@@ -9809,19 +9845,18 @@
         <v/>
       </c>
       <c r="J7" s="18">
-        <f>DATE(YEAR($E$3),MONTH($E$3),1)</f>
+        <f>IF(ISNUMBER($H$3),$H$3,DATE(YEAR(K7),MONTH(K7),1))</f>
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>$E$3</f>
+        <f>IF(ISNUMBER($J$3),$J$3,$E$3)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>Прошлый, те же дни</t>
-        </is>
+      <c r="A8" s="19">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Предыдущий, той же длины","Прошлый, те же дни")</f>
+        <v/>
       </c>
       <c r="B8" s="20">
         <f>SUMIFS('Данные'!$C:$C,'Данные'!$A:$A,"&gt;="&amp;$J$8,'Данные'!$A:$A,"&lt;"&amp;$K$8+1,'Данные'!$B:$B,$B$3)</f>
@@ -9856,11 +9891,11 @@
         <v/>
       </c>
       <c r="J8" s="25">
-        <f>IF(FALSE,2*J7-K7-1,EDATE(J7,-1))</f>
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),2*J7-K7-1,EDATE(J7,-1))</f>
         <v/>
       </c>
       <c r="K8" s="25">
-        <f>IF(FALSE,J7-1,EDATE(K7,-1))</f>
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),J7-1,EDATE(K7,-1))</f>
         <v/>
       </c>
     </row>
@@ -13448,6 +13483,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H3 J3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Период" prompt="Дата. Пусто — текущий месяц." type="date" operator="greaterThan">
+      <formula1>1</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -13584,17 +13624,34 @@
         <f>'⚙ Настройки'!$B$7</f>
         <v/>
       </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Период с</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>по</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="n"/>
       <c r="M3" s="9" t="inlineStr">
         <is>
           <t>📈 По дням, последние 90</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="H4" s="10">
+        <f>IF(AND(ISNUMBER(H3),ISNUMBER(J3),H3&gt;J3),"⚠ Дата «с» позже даты «по»",IF(OR(ISNUMBER(H3),ISNUMBER(J3)),"Сравнение — с предыдущим периодом той же длины. Очистите поля, чтобы вернуть текущий месяц.","Пусто — текущий месяц. Дату выбирают двойным щелчком."))</f>
+        <v/>
+      </c>
+    </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Этот месяц против тех же дней прошлого</t>
-        </is>
+      <c r="A5" s="9">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Выбранный период против предыдущего той же длины","Этот месяц против тех же дней прошлого")</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -13655,10 +13712,9 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Этот месяц</t>
-        </is>
+      <c r="A7" s="12">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Выбранный период","Этот месяц")</f>
+        <v/>
       </c>
       <c r="B7" s="13">
         <f>SUMIFS('Данные'!$C:$C,'Данные'!$A:$A,"&gt;="&amp;$J$7,'Данные'!$A:$A,"&lt;"&amp;$K$7+1,'Данные'!$B:$B,$B$3)</f>
@@ -13693,19 +13749,18 @@
         <v/>
       </c>
       <c r="J7" s="18">
-        <f>DATE(YEAR($E$3),MONTH($E$3),1)</f>
+        <f>IF(ISNUMBER($H$3),$H$3,DATE(YEAR(K7),MONTH(K7),1))</f>
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>$E$3</f>
+        <f>IF(ISNUMBER($J$3),$J$3,$E$3)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>Прошлый, те же дни</t>
-        </is>
+      <c r="A8" s="19">
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),"Предыдущий, той же длины","Прошлый, те же дни")</f>
+        <v/>
       </c>
       <c r="B8" s="20">
         <f>SUMIFS('Данные'!$C:$C,'Данные'!$A:$A,"&gt;="&amp;$J$8,'Данные'!$A:$A,"&lt;"&amp;$K$8+1,'Данные'!$B:$B,$B$3)</f>
@@ -13740,11 +13795,11 @@
         <v/>
       </c>
       <c r="J8" s="25">
-        <f>IF(FALSE,2*J7-K7-1,EDATE(J7,-1))</f>
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),2*J7-K7-1,EDATE(J7,-1))</f>
         <v/>
       </c>
       <c r="K8" s="25">
-        <f>IF(FALSE,J7-1,EDATE(K7,-1))</f>
+        <f>IF(OR(ISNUMBER($H$3),ISNUMBER($J$3)),J7-1,EDATE(K7,-1))</f>
         <v/>
       </c>
     </row>
@@ -17332,6 +17387,11 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H3 J3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Период" prompt="Дата. Пусто — текущий месяц." type="date" operator="greaterThan">
+      <formula1>1</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Chart spend next to subscriptions for the same periods
The summary pairs subscriptions and spend by week and by month, with a
trendline on each, so their dynamics can be compared side by side.
Direction sheets pair daily subscriptions and spend; cost per
subscription moves to the row below.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kPBSYq9ZY5XtdXkATthy6
</commit_message>
<xml_diff>
--- a/sova-report/sova-report.xlsx
+++ b/sova-report/sova-report.xlsx
@@ -575,6 +575,507 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Подписки по дням (пунктир — тренд)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Направление 2'!G12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1BAF7A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <trendline>
+            <spPr>
+              <a:ln w="22000">
+                <a:solidFill>
+                  <a:srgbClr val="1F2A44"/>
+                </a:solidFill>
+                <a:prstDash val="dash"/>
+              </a:ln>
+            </spPr>
+            <trendlineType val="linear"/>
+            <dispRSqr val="0"/>
+            <dispEq val="0"/>
+          </trendline>
+          <cat>
+            <numRef>
+              <f>'Направление 2'!$A$13:$A$102</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Направление 2'!$G$13:$G$102</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Расход по дням, ₽ (пунктир — тренд)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Направление 2'!B12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <trendline>
+            <spPr>
+              <a:ln w="22000">
+                <a:solidFill>
+                  <a:srgbClr val="1F2A44"/>
+                </a:solidFill>
+                <a:prstDash val="dash"/>
+              </a:ln>
+            </spPr>
+            <trendlineType val="linear"/>
+            <dispRSqr val="0"/>
+            <dispEq val="0"/>
+          </trendline>
+          <cat>
+            <numRef>
+              <f>'Направление 2'!$A$13:$A$102</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Направление 2'!$B$13:$B$102</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Цена подписки по дням, ₽</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Направление 2'!H12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Направление 2'!$A$13:$A$102</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Направление 2'!$H$13:$H$102</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Подписки по дням (пунктир — тренд)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Направление 3'!G12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1BAF7A"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <trendline>
+            <spPr>
+              <a:ln w="22000">
+                <a:solidFill>
+                  <a:srgbClr val="1F2A44"/>
+                </a:solidFill>
+                <a:prstDash val="dash"/>
+              </a:ln>
+            </spPr>
+            <trendlineType val="linear"/>
+            <dispRSqr val="0"/>
+            <dispEq val="0"/>
+          </trendline>
+          <cat>
+            <numRef>
+              <f>'Направление 3'!$A$13:$A$102</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Направление 3'!$G$13:$G$102</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Расход по дням, ₽ (пунктир — тренд)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Направление 3'!B12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <trendline>
+            <spPr>
+              <a:ln w="22000">
+                <a:solidFill>
+                  <a:srgbClr val="1F2A44"/>
+                </a:solidFill>
+                <a:prstDash val="dash"/>
+              </a:ln>
+            </spPr>
+            <trendlineType val="linear"/>
+            <dispRSqr val="0"/>
+            <dispEq val="0"/>
+          </trendline>
+          <cat>
+            <numRef>
+              <f>'Направление 3'!$A$13:$A$102</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Направление 3'!$B$13:$B$102</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Цена подписки по дням, ₽</a:t>
             </a:r>
           </a:p>
@@ -656,6 +1157,108 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Расход по неделям — вся клиника, ₽ (пунктир — тренд)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Сводная'!E77</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <trendline>
+            <spPr>
+              <a:ln w="22000">
+                <a:solidFill>
+                  <a:srgbClr val="1F2A44"/>
+                </a:solidFill>
+                <a:prstDash val="dash"/>
+              </a:ln>
+            </spPr>
+            <trendlineType val="linear"/>
+            <dispRSqr val="0"/>
+            <dispEq val="0"/>
+          </trendline>
+          <cat>
+            <numRef>
+              <f>'Сводная'!$A$78:$A$103</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Сводная'!$E$78:$E$103</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -757,7 +1360,109 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Расход по месяцам — вся клиника, ₽ (пунктир — тренд)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Сводная'!E136</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <trendline>
+            <spPr>
+              <a:ln w="22000">
+                <a:solidFill>
+                  <a:srgbClr val="1F2A44"/>
+                </a:solidFill>
+                <a:prstDash val="dash"/>
+              </a:ln>
+            </spPr>
+            <trendlineType val="linear"/>
+            <dispRSqr val="0"/>
+            <dispEq val="0"/>
+          </trendline>
+          <cat>
+            <numRef>
+              <f>'Сводная'!$A$137:$A$148</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Сводная'!$E$137:$E$148</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -925,7 +1630,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -1093,7 +1798,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -1195,7 +1900,109 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Расход по дням, ₽ (пунктир — тренд)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Направление 1'!B12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <trendline>
+            <spPr>
+              <a:ln w="22000">
+                <a:solidFill>
+                  <a:srgbClr val="1F2A44"/>
+                </a:solidFill>
+                <a:prstDash val="dash"/>
+              </a:ln>
+            </spPr>
+            <trendlineType val="linear"/>
+            <dispRSqr val="0"/>
+            <dispEq val="0"/>
+          </trendline>
+          <cat>
+            <numRef>
+              <f>'Направление 1'!$A$13:$A$102</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Направление 1'!$B$13:$B$102</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
@@ -1256,303 +2063,6 @@
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Подписки по дням (пунктир — тренд)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Направление 2'!G12</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1BAF7A"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="1BAF7A"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <trendline>
-            <spPr>
-              <a:ln w="22000">
-                <a:solidFill>
-                  <a:srgbClr val="1F2A44"/>
-                </a:solidFill>
-                <a:prstDash val="dash"/>
-              </a:ln>
-            </spPr>
-            <trendlineType val="linear"/>
-            <dispRSqr val="0"/>
-            <dispEq val="0"/>
-          </trendline>
-          <cat>
-            <numRef>
-              <f>'Направление 2'!$A$13:$A$102</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Направление 2'!$G$13:$G$102</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="40"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Цена подписки по дням, ₽</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Направление 2'!H12</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="22000">
-              <a:solidFill>
-                <a:srgbClr val="EB6834"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Направление 2'!$A$13:$A$102</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Направление 2'!$H$13:$H$102</f>
-            </numRef>
-          </val>
-          <smooth val="0"/>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Подписки по дням (пунктир — тренд)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Направление 3'!G12</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1BAF7A"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="1BAF7A"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <trendline>
-            <spPr>
-              <a:ln w="22000">
-                <a:solidFill>
-                  <a:srgbClr val="1F2A44"/>
-                </a:solidFill>
-                <a:prstDash val="dash"/>
-              </a:ln>
-            </spPr>
-            <trendlineType val="linear"/>
-            <dispRSqr val="0"/>
-            <dispEq val="0"/>
-          </trendline>
-          <cat>
-            <numRef>
-              <f>'Направление 3'!$A$13:$A$102</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Направление 3'!$G$13:$G$102</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="40"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -1675,6 +2185,50 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5328000" cy="2664000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5328000" cy="2664000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1719,6 +2273,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5328000" cy="2664000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1773,6 +2349,28 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5328000" cy="2664000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1817,6 +2415,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5328000" cy="2664000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2251,7 +2871,7 @@
       <c r="J3" s="8" t="n"/>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>📈 Тенденция подписок по неделям и месяцам (завершённые периоды)</t>
+          <t>📈 Подписки и расход по неделям и месяцам (завершённые периоды)</t>
         </is>
       </c>
     </row>
@@ -5830,7 +6450,7 @@
       <c r="J3" s="8" t="n"/>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>📈 По дням, последние 90</t>
+          <t>📈 Подписки и расход по дням, последние 90</t>
         </is>
       </c>
     </row>
@@ -9734,7 +10354,7 @@
       <c r="J3" s="8" t="n"/>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>📈 По дням, последние 90</t>
+          <t>📈 Подписки и расход по дням, последние 90</t>
         </is>
       </c>
     </row>
@@ -13638,7 +14258,7 @@
       <c r="J3" s="8" t="n"/>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>📈 По дням, последние 90</t>
+          <t>📈 Подписки и расход по дням, последние 90</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stack charts in one column next to the tables
The right-hand chart column sat beyond the visible area, so the daily
spend chart looked missing. All charts now stack in one column right of
the tables, with spend directly under subscriptions for the same periods.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kPBSYq9ZY5XtdXkATthy6
</commit_message>
<xml_diff>
--- a/sova-report/sova-report.xlsx
+++ b/sova-report/sova-report.xlsx
@@ -2121,9 +2121,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>12</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2145,7 +2145,7 @@
     <from>
       <col>12</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2165,9 +2165,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>12</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>48</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2189,7 +2189,7 @@
     <from>
       <col>12</col>
       <colOff>0</colOff>
-      <row>33</row>
+      <row>63</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2209,9 +2209,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>12</col>
       <colOff>0</colOff>
-      <row>33</row>
+      <row>78</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2258,9 +2258,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>12</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2282,7 +2282,7 @@
     <from>
       <col>12</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2329,9 +2329,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>12</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2353,7 +2353,7 @@
     <from>
       <col>12</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2400,9 +2400,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>12</col>
       <colOff>0</colOff>
-      <row>3</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>
@@ -2424,7 +2424,7 @@
     <from>
       <col>12</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5328000" cy="2664000"/>

</xml_diff>

<commit_message>
Keep the full history of weeks and months, labelled with the year
Weekly and monthly tables on the summary and direction sheets no longer
drop old periods after 26 weeks and 12 months; they keep everything
since TRENDS_FROM (with a ten-year safety cap). Labels now carry the
year so periods from different years stay distinct. Checked against
50 and 100 weeks of data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kPBSYq9ZY5XtdXkATthy6
</commit_message>
<xml_diff>
--- a/sova-report/sova-report.xlsx
+++ b/sova-report/sova-report.xlsx
@@ -3370,7 +3370,7 @@
     </row>
     <row r="20">
       <c r="A20" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B20" s="31">
@@ -3393,7 +3393,7 @@
     </row>
     <row r="21">
       <c r="A21" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B21" s="38">
@@ -3419,7 +3419,7 @@
     </row>
     <row r="22">
       <c r="A22" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B22" s="31">
@@ -3445,7 +3445,7 @@
     </row>
     <row r="23">
       <c r="A23" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B23" s="38">
@@ -3471,7 +3471,7 @@
     </row>
     <row r="24">
       <c r="A24" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B24" s="31">
@@ -3497,7 +3497,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B25" s="38">
@@ -3523,7 +3523,7 @@
     </row>
     <row r="26">
       <c r="A26" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B26" s="31">
@@ -3549,7 +3549,7 @@
     </row>
     <row r="27">
       <c r="A27" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B27" s="38">
@@ -3575,7 +3575,7 @@
     </row>
     <row r="28">
       <c r="A28" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B28" s="31">
@@ -3601,7 +3601,7 @@
     </row>
     <row r="29">
       <c r="A29" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B29" s="38">
@@ -3627,7 +3627,7 @@
     </row>
     <row r="30">
       <c r="A30" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B30" s="31">
@@ -3653,7 +3653,7 @@
     </row>
     <row r="31">
       <c r="A31" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B31" s="38">
@@ -3679,7 +3679,7 @@
     </row>
     <row r="32">
       <c r="A32" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B32" s="31">
@@ -3705,7 +3705,7 @@
     </row>
     <row r="33">
       <c r="A33" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B33" s="38">
@@ -3731,7 +3731,7 @@
     </row>
     <row r="34">
       <c r="A34" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B34" s="31">
@@ -3757,7 +3757,7 @@
     </row>
     <row r="35">
       <c r="A35" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B35" s="38">
@@ -3783,7 +3783,7 @@
     </row>
     <row r="36">
       <c r="A36" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B36" s="31">
@@ -3809,7 +3809,7 @@
     </row>
     <row r="37">
       <c r="A37" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B37" s="38">
@@ -3835,7 +3835,7 @@
     </row>
     <row r="38">
       <c r="A38" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B38" s="31">
@@ -3861,7 +3861,7 @@
     </row>
     <row r="39">
       <c r="A39" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B39" s="38">
@@ -3887,7 +3887,7 @@
     </row>
     <row r="40">
       <c r="A40" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B40" s="31">
@@ -3913,7 +3913,7 @@
     </row>
     <row r="41">
       <c r="A41" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B41" s="38">
@@ -3939,7 +3939,7 @@
     </row>
     <row r="42">
       <c r="A42" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B42" s="31">
@@ -3965,7 +3965,7 @@
     </row>
     <row r="43">
       <c r="A43" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B43" s="38">
@@ -3991,7 +3991,7 @@
     </row>
     <row r="44">
       <c r="A44" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B44" s="31">
@@ -4017,7 +4017,7 @@
     </row>
     <row r="45">
       <c r="A45" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B45" s="38">
@@ -4074,7 +4074,7 @@
     </row>
     <row r="49">
       <c r="A49" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B49" s="33">
@@ -4096,7 +4096,7 @@
     </row>
     <row r="50">
       <c r="A50" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B50" s="40">
@@ -4118,7 +4118,7 @@
     </row>
     <row r="51">
       <c r="A51" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B51" s="33">
@@ -4140,7 +4140,7 @@
     </row>
     <row r="52">
       <c r="A52" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B52" s="40">
@@ -4162,7 +4162,7 @@
     </row>
     <row r="53">
       <c r="A53" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B53" s="33">
@@ -4184,7 +4184,7 @@
     </row>
     <row r="54">
       <c r="A54" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B54" s="40">
@@ -4206,7 +4206,7 @@
     </row>
     <row r="55">
       <c r="A55" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B55" s="33">
@@ -4228,7 +4228,7 @@
     </row>
     <row r="56">
       <c r="A56" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B56" s="40">
@@ -4250,7 +4250,7 @@
     </row>
     <row r="57">
       <c r="A57" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B57" s="33">
@@ -4272,7 +4272,7 @@
     </row>
     <row r="58">
       <c r="A58" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B58" s="40">
@@ -4294,7 +4294,7 @@
     </row>
     <row r="59">
       <c r="A59" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B59" s="33">
@@ -4316,7 +4316,7 @@
     </row>
     <row r="60">
       <c r="A60" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B60" s="40">
@@ -4338,7 +4338,7 @@
     </row>
     <row r="61">
       <c r="A61" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B61" s="33">
@@ -4360,7 +4360,7 @@
     </row>
     <row r="62">
       <c r="A62" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B62" s="40">
@@ -4382,7 +4382,7 @@
     </row>
     <row r="63">
       <c r="A63" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B63" s="33">
@@ -4404,7 +4404,7 @@
     </row>
     <row r="64">
       <c r="A64" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B64" s="40">
@@ -4426,7 +4426,7 @@
     </row>
     <row r="65">
       <c r="A65" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B65" s="33">
@@ -4448,7 +4448,7 @@
     </row>
     <row r="66">
       <c r="A66" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B66" s="40">
@@ -4470,7 +4470,7 @@
     </row>
     <row r="67">
       <c r="A67" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B67" s="33">
@@ -4492,7 +4492,7 @@
     </row>
     <row r="68">
       <c r="A68" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B68" s="40">
@@ -4514,7 +4514,7 @@
     </row>
     <row r="69">
       <c r="A69" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B69" s="33">
@@ -4536,7 +4536,7 @@
     </row>
     <row r="70">
       <c r="A70" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B70" s="40">
@@ -4558,7 +4558,7 @@
     </row>
     <row r="71">
       <c r="A71" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B71" s="33">
@@ -4580,7 +4580,7 @@
     </row>
     <row r="72">
       <c r="A72" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B72" s="40">
@@ -4602,7 +4602,7 @@
     </row>
     <row r="73">
       <c r="A73" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B73" s="33">
@@ -4624,7 +4624,7 @@
     </row>
     <row r="74">
       <c r="A74" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B74" s="40">
@@ -4677,7 +4677,7 @@
     </row>
     <row r="78">
       <c r="A78" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B78" s="30">
@@ -4699,7 +4699,7 @@
     </row>
     <row r="79">
       <c r="A79" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B79" s="37">
@@ -4721,7 +4721,7 @@
     </row>
     <row r="80">
       <c r="A80" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B80" s="30">
@@ -4743,7 +4743,7 @@
     </row>
     <row r="81">
       <c r="A81" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B81" s="37">
@@ -4765,7 +4765,7 @@
     </row>
     <row r="82">
       <c r="A82" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B82" s="30">
@@ -4787,7 +4787,7 @@
     </row>
     <row r="83">
       <c r="A83" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B83" s="37">
@@ -4809,7 +4809,7 @@
     </row>
     <row r="84">
       <c r="A84" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B84" s="30">
@@ -4831,7 +4831,7 @@
     </row>
     <row r="85">
       <c r="A85" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B85" s="37">
@@ -4853,7 +4853,7 @@
     </row>
     <row r="86">
       <c r="A86" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B86" s="30">
@@ -4875,7 +4875,7 @@
     </row>
     <row r="87">
       <c r="A87" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B87" s="37">
@@ -4897,7 +4897,7 @@
     </row>
     <row r="88">
       <c r="A88" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B88" s="30">
@@ -4919,7 +4919,7 @@
     </row>
     <row r="89">
       <c r="A89" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B89" s="37">
@@ -4941,7 +4941,7 @@
     </row>
     <row r="90">
       <c r="A90" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B90" s="30">
@@ -4963,7 +4963,7 @@
     </row>
     <row r="91">
       <c r="A91" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B91" s="37">
@@ -4985,7 +4985,7 @@
     </row>
     <row r="92">
       <c r="A92" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B92" s="30">
@@ -5007,7 +5007,7 @@
     </row>
     <row r="93">
       <c r="A93" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B93" s="37">
@@ -5029,7 +5029,7 @@
     </row>
     <row r="94">
       <c r="A94" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B94" s="30">
@@ -5051,7 +5051,7 @@
     </row>
     <row r="95">
       <c r="A95" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B95" s="37">
@@ -5073,7 +5073,7 @@
     </row>
     <row r="96">
       <c r="A96" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B96" s="30">
@@ -5095,7 +5095,7 @@
     </row>
     <row r="97">
       <c r="A97" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B97" s="37">
@@ -5117,7 +5117,7 @@
     </row>
     <row r="98">
       <c r="A98" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B98" s="30">
@@ -5139,7 +5139,7 @@
     </row>
     <row r="99">
       <c r="A99" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B99" s="37">
@@ -5161,7 +5161,7 @@
     </row>
     <row r="100">
       <c r="A100" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B100" s="30">
@@ -5183,7 +5183,7 @@
     </row>
     <row r="101">
       <c r="A101" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B101" s="37">
@@ -5205,7 +5205,7 @@
     </row>
     <row r="102">
       <c r="A102" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B102" s="30">
@@ -5227,7 +5227,7 @@
     </row>
     <row r="103">
       <c r="A103" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B103" s="37">
@@ -5299,7 +5299,7 @@
     </row>
     <row r="107">
       <c r="A107" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11))</f>
         <v/>
       </c>
       <c r="B107" s="31">
@@ -5322,7 +5322,7 @@
     </row>
     <row r="108">
       <c r="A108" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10))</f>
         <v/>
       </c>
       <c r="B108" s="38">
@@ -5348,7 +5348,7 @@
     </row>
     <row r="109">
       <c r="A109" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9))</f>
         <v/>
       </c>
       <c r="B109" s="31">
@@ -5374,7 +5374,7 @@
     </row>
     <row r="110">
       <c r="A110" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8))</f>
         <v/>
       </c>
       <c r="B110" s="38">
@@ -5400,7 +5400,7 @@
     </row>
     <row r="111">
       <c r="A111" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7))</f>
         <v/>
       </c>
       <c r="B111" s="31">
@@ -5426,7 +5426,7 @@
     </row>
     <row r="112">
       <c r="A112" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6))</f>
         <v/>
       </c>
       <c r="B112" s="38">
@@ -5452,7 +5452,7 @@
     </row>
     <row r="113">
       <c r="A113" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5))</f>
         <v/>
       </c>
       <c r="B113" s="31">
@@ -5478,7 +5478,7 @@
     </row>
     <row r="114">
       <c r="A114" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4))</f>
         <v/>
       </c>
       <c r="B114" s="38">
@@ -5504,7 +5504,7 @@
     </row>
     <row r="115">
       <c r="A115" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3))</f>
         <v/>
       </c>
       <c r="B115" s="31">
@@ -5530,7 +5530,7 @@
     </row>
     <row r="116">
       <c r="A116" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2))</f>
         <v/>
       </c>
       <c r="B116" s="38">
@@ -5556,7 +5556,7 @@
     </row>
     <row r="117">
       <c r="A117" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1))</f>
         <v/>
       </c>
       <c r="B117" s="31">
@@ -5582,7 +5582,7 @@
     </row>
     <row r="118">
       <c r="A118" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0))</f>
         <v/>
       </c>
       <c r="B118" s="38">
@@ -5639,7 +5639,7 @@
     </row>
     <row r="122">
       <c r="A122" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11))</f>
         <v/>
       </c>
       <c r="B122" s="33">
@@ -5661,7 +5661,7 @@
     </row>
     <row r="123">
       <c r="A123" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10))</f>
         <v/>
       </c>
       <c r="B123" s="40">
@@ -5683,7 +5683,7 @@
     </row>
     <row r="124">
       <c r="A124" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9))</f>
         <v/>
       </c>
       <c r="B124" s="33">
@@ -5705,7 +5705,7 @@
     </row>
     <row r="125">
       <c r="A125" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8))</f>
         <v/>
       </c>
       <c r="B125" s="40">
@@ -5727,7 +5727,7 @@
     </row>
     <row r="126">
       <c r="A126" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7))</f>
         <v/>
       </c>
       <c r="B126" s="33">
@@ -5749,7 +5749,7 @@
     </row>
     <row r="127">
       <c r="A127" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6))</f>
         <v/>
       </c>
       <c r="B127" s="40">
@@ -5771,7 +5771,7 @@
     </row>
     <row r="128">
       <c r="A128" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5))</f>
         <v/>
       </c>
       <c r="B128" s="33">
@@ -5793,7 +5793,7 @@
     </row>
     <row r="129">
       <c r="A129" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4))</f>
         <v/>
       </c>
       <c r="B129" s="40">
@@ -5815,7 +5815,7 @@
     </row>
     <row r="130">
       <c r="A130" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3))</f>
         <v/>
       </c>
       <c r="B130" s="33">
@@ -5837,7 +5837,7 @@
     </row>
     <row r="131">
       <c r="A131" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2))</f>
         <v/>
       </c>
       <c r="B131" s="40">
@@ -5859,7 +5859,7 @@
     </row>
     <row r="132">
       <c r="A132" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1))</f>
         <v/>
       </c>
       <c r="B132" s="33">
@@ -5881,7 +5881,7 @@
     </row>
     <row r="133">
       <c r="A133" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0))</f>
         <v/>
       </c>
       <c r="B133" s="40">
@@ -5934,7 +5934,7 @@
     </row>
     <row r="137">
       <c r="A137" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11))</f>
         <v/>
       </c>
       <c r="B137" s="30">
@@ -5956,7 +5956,7 @@
     </row>
     <row r="138">
       <c r="A138" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10))</f>
         <v/>
       </c>
       <c r="B138" s="37">
@@ -5978,7 +5978,7 @@
     </row>
     <row r="139">
       <c r="A139" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9))</f>
         <v/>
       </c>
       <c r="B139" s="30">
@@ -6000,7 +6000,7 @@
     </row>
     <row r="140">
       <c r="A140" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8))</f>
         <v/>
       </c>
       <c r="B140" s="37">
@@ -6022,7 +6022,7 @@
     </row>
     <row r="141">
       <c r="A141" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7))</f>
         <v/>
       </c>
       <c r="B141" s="30">
@@ -6044,7 +6044,7 @@
     </row>
     <row r="142">
       <c r="A142" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6))</f>
         <v/>
       </c>
       <c r="B142" s="37">
@@ -6066,7 +6066,7 @@
     </row>
     <row r="143">
       <c r="A143" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5))</f>
         <v/>
       </c>
       <c r="B143" s="30">
@@ -6088,7 +6088,7 @@
     </row>
     <row r="144">
       <c r="A144" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4))</f>
         <v/>
       </c>
       <c r="B144" s="37">
@@ -6110,7 +6110,7 @@
     </row>
     <row r="145">
       <c r="A145" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3))</f>
         <v/>
       </c>
       <c r="B145" s="30">
@@ -6132,7 +6132,7 @@
     </row>
     <row r="146">
       <c r="A146" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2))</f>
         <v/>
       </c>
       <c r="B146" s="37">
@@ -6154,7 +6154,7 @@
     </row>
     <row r="147">
       <c r="A147" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1))</f>
         <v/>
       </c>
       <c r="B147" s="30">
@@ -6176,7 +6176,7 @@
     </row>
     <row r="148">
       <c r="A148" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0))</f>
         <v/>
       </c>
       <c r="B148" s="37">
@@ -6726,7 +6726,7 @@
     </row>
     <row r="13">
       <c r="A13" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B13" s="30">
@@ -6764,7 +6764,7 @@
     </row>
     <row r="14">
       <c r="A14" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B14" s="37">
@@ -6802,7 +6802,7 @@
     </row>
     <row r="15">
       <c r="A15" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B15" s="30">
@@ -6840,7 +6840,7 @@
     </row>
     <row r="16">
       <c r="A16" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B16" s="37">
@@ -6878,7 +6878,7 @@
     </row>
     <row r="17">
       <c r="A17" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B17" s="30">
@@ -6916,7 +6916,7 @@
     </row>
     <row r="18">
       <c r="A18" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B18" s="37">
@@ -6954,7 +6954,7 @@
     </row>
     <row r="19">
       <c r="A19" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B19" s="30">
@@ -6992,7 +6992,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B20" s="37">
@@ -7030,7 +7030,7 @@
     </row>
     <row r="21">
       <c r="A21" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B21" s="30">
@@ -7068,7 +7068,7 @@
     </row>
     <row r="22">
       <c r="A22" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B22" s="37">
@@ -7106,7 +7106,7 @@
     </row>
     <row r="23">
       <c r="A23" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B23" s="30">
@@ -7144,7 +7144,7 @@
     </row>
     <row r="24">
       <c r="A24" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B24" s="37">
@@ -7182,7 +7182,7 @@
     </row>
     <row r="25">
       <c r="A25" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B25" s="30">
@@ -7220,7 +7220,7 @@
     </row>
     <row r="26">
       <c r="A26" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B26" s="37">
@@ -7258,7 +7258,7 @@
     </row>
     <row r="27">
       <c r="A27" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B27" s="30">
@@ -7296,7 +7296,7 @@
     </row>
     <row r="28">
       <c r="A28" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B28" s="37">
@@ -7334,7 +7334,7 @@
     </row>
     <row r="29">
       <c r="A29" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B29" s="30">
@@ -7372,7 +7372,7 @@
     </row>
     <row r="30">
       <c r="A30" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B30" s="37">
@@ -7410,7 +7410,7 @@
     </row>
     <row r="31">
       <c r="A31" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B31" s="30">
@@ -7448,7 +7448,7 @@
     </row>
     <row r="32">
       <c r="A32" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B32" s="37">
@@ -7486,7 +7486,7 @@
     </row>
     <row r="33">
       <c r="A33" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B33" s="30">
@@ -7524,7 +7524,7 @@
     </row>
     <row r="34">
       <c r="A34" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B34" s="37">
@@ -7562,7 +7562,7 @@
     </row>
     <row r="35">
       <c r="A35" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B35" s="30">
@@ -7600,7 +7600,7 @@
     </row>
     <row r="36">
       <c r="A36" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B36" s="37">
@@ -7638,7 +7638,7 @@
     </row>
     <row r="37">
       <c r="A37" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B37" s="30">
@@ -7676,7 +7676,7 @@
     </row>
     <row r="38">
       <c r="A38" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B38" s="37">
@@ -7807,7 +7807,7 @@
     </row>
     <row r="43">
       <c r="A43" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11))</f>
         <v/>
       </c>
       <c r="B43" s="30">
@@ -7845,7 +7845,7 @@
     </row>
     <row r="44">
       <c r="A44" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10))</f>
         <v/>
       </c>
       <c r="B44" s="37">
@@ -7883,7 +7883,7 @@
     </row>
     <row r="45">
       <c r="A45" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9))</f>
         <v/>
       </c>
       <c r="B45" s="30">
@@ -7921,7 +7921,7 @@
     </row>
     <row r="46">
       <c r="A46" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8))</f>
         <v/>
       </c>
       <c r="B46" s="37">
@@ -7959,7 +7959,7 @@
     </row>
     <row r="47">
       <c r="A47" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7))</f>
         <v/>
       </c>
       <c r="B47" s="30">
@@ -7997,7 +7997,7 @@
     </row>
     <row r="48">
       <c r="A48" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6))</f>
         <v/>
       </c>
       <c r="B48" s="37">
@@ -8035,7 +8035,7 @@
     </row>
     <row r="49">
       <c r="A49" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5))</f>
         <v/>
       </c>
       <c r="B49" s="30">
@@ -8073,7 +8073,7 @@
     </row>
     <row r="50">
       <c r="A50" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4))</f>
         <v/>
       </c>
       <c r="B50" s="37">
@@ -8111,7 +8111,7 @@
     </row>
     <row r="51">
       <c r="A51" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3))</f>
         <v/>
       </c>
       <c r="B51" s="30">
@@ -8149,7 +8149,7 @@
     </row>
     <row r="52">
       <c r="A52" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2))</f>
         <v/>
       </c>
       <c r="B52" s="37">
@@ -8187,7 +8187,7 @@
     </row>
     <row r="53">
       <c r="A53" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1))</f>
         <v/>
       </c>
       <c r="B53" s="30">
@@ -8225,7 +8225,7 @@
     </row>
     <row r="54">
       <c r="A54" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0))</f>
         <v/>
       </c>
       <c r="B54" s="37">
@@ -12359,7 +12359,7 @@
     </row>
     <row r="13">
       <c r="A13" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B13" s="30">
@@ -12397,7 +12397,7 @@
     </row>
     <row r="14">
       <c r="A14" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B14" s="37">
@@ -12435,7 +12435,7 @@
     </row>
     <row r="15">
       <c r="A15" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B15" s="30">
@@ -12473,7 +12473,7 @@
     </row>
     <row r="16">
       <c r="A16" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B16" s="37">
@@ -12511,7 +12511,7 @@
     </row>
     <row r="17">
       <c r="A17" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B17" s="30">
@@ -12549,7 +12549,7 @@
     </row>
     <row r="18">
       <c r="A18" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B18" s="37">
@@ -12587,7 +12587,7 @@
     </row>
     <row r="19">
       <c r="A19" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B19" s="30">
@@ -12625,7 +12625,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B20" s="37">
@@ -12663,7 +12663,7 @@
     </row>
     <row r="21">
       <c r="A21" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B21" s="30">
@@ -12701,7 +12701,7 @@
     </row>
     <row r="22">
       <c r="A22" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B22" s="37">
@@ -12739,7 +12739,7 @@
     </row>
     <row r="23">
       <c r="A23" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B23" s="30">
@@ -12777,7 +12777,7 @@
     </row>
     <row r="24">
       <c r="A24" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B24" s="37">
@@ -12815,7 +12815,7 @@
     </row>
     <row r="25">
       <c r="A25" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B25" s="30">
@@ -12853,7 +12853,7 @@
     </row>
     <row r="26">
       <c r="A26" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B26" s="37">
@@ -12891,7 +12891,7 @@
     </row>
     <row r="27">
       <c r="A27" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B27" s="30">
@@ -12929,7 +12929,7 @@
     </row>
     <row r="28">
       <c r="A28" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B28" s="37">
@@ -12967,7 +12967,7 @@
     </row>
     <row r="29">
       <c r="A29" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B29" s="30">
@@ -13005,7 +13005,7 @@
     </row>
     <row r="30">
       <c r="A30" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B30" s="37">
@@ -13043,7 +13043,7 @@
     </row>
     <row r="31">
       <c r="A31" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B31" s="30">
@@ -13081,7 +13081,7 @@
     </row>
     <row r="32">
       <c r="A32" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B32" s="37">
@@ -13119,7 +13119,7 @@
     </row>
     <row r="33">
       <c r="A33" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B33" s="30">
@@ -13157,7 +13157,7 @@
     </row>
     <row r="34">
       <c r="A34" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B34" s="37">
@@ -13195,7 +13195,7 @@
     </row>
     <row r="35">
       <c r="A35" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B35" s="30">
@@ -13233,7 +13233,7 @@
     </row>
     <row r="36">
       <c r="A36" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B36" s="37">
@@ -13271,7 +13271,7 @@
     </row>
     <row r="37">
       <c r="A37" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B37" s="30">
@@ -13309,7 +13309,7 @@
     </row>
     <row r="38">
       <c r="A38" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B38" s="37">
@@ -13440,7 +13440,7 @@
     </row>
     <row r="43">
       <c r="A43" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11))</f>
         <v/>
       </c>
       <c r="B43" s="30">
@@ -13478,7 +13478,7 @@
     </row>
     <row r="44">
       <c r="A44" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10))</f>
         <v/>
       </c>
       <c r="B44" s="37">
@@ -13516,7 +13516,7 @@
     </row>
     <row r="45">
       <c r="A45" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9))</f>
         <v/>
       </c>
       <c r="B45" s="30">
@@ -13554,7 +13554,7 @@
     </row>
     <row r="46">
       <c r="A46" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8))</f>
         <v/>
       </c>
       <c r="B46" s="37">
@@ -13592,7 +13592,7 @@
     </row>
     <row r="47">
       <c r="A47" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7))</f>
         <v/>
       </c>
       <c r="B47" s="30">
@@ -13630,7 +13630,7 @@
     </row>
     <row r="48">
       <c r="A48" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6))</f>
         <v/>
       </c>
       <c r="B48" s="37">
@@ -13668,7 +13668,7 @@
     </row>
     <row r="49">
       <c r="A49" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5))</f>
         <v/>
       </c>
       <c r="B49" s="30">
@@ -13706,7 +13706,7 @@
     </row>
     <row r="50">
       <c r="A50" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4))</f>
         <v/>
       </c>
       <c r="B50" s="37">
@@ -13744,7 +13744,7 @@
     </row>
     <row r="51">
       <c r="A51" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3))</f>
         <v/>
       </c>
       <c r="B51" s="30">
@@ -13782,7 +13782,7 @@
     </row>
     <row r="52">
       <c r="A52" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2))</f>
         <v/>
       </c>
       <c r="B52" s="37">
@@ -13820,7 +13820,7 @@
     </row>
     <row r="53">
       <c r="A53" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1))</f>
         <v/>
       </c>
       <c r="B53" s="30">
@@ -13858,7 +13858,7 @@
     </row>
     <row r="54">
       <c r="A54" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0))</f>
         <v/>
       </c>
       <c r="B54" s="37">
@@ -17992,7 +17992,7 @@
     </row>
     <row r="13">
       <c r="A13" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*25)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B13" s="30">
@@ -18030,7 +18030,7 @@
     </row>
     <row r="14">
       <c r="A14" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*24)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B14" s="37">
@@ -18068,7 +18068,7 @@
     </row>
     <row r="15">
       <c r="A15" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*23)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B15" s="30">
@@ -18106,7 +18106,7 @@
     </row>
     <row r="16">
       <c r="A16" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*22)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B16" s="37">
@@ -18144,7 +18144,7 @@
     </row>
     <row r="17">
       <c r="A17" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*21)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B17" s="30">
@@ -18182,7 +18182,7 @@
     </row>
     <row r="18">
       <c r="A18" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*20)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B18" s="37">
@@ -18220,7 +18220,7 @@
     </row>
     <row r="19">
       <c r="A19" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*19)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B19" s="30">
@@ -18258,7 +18258,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*18)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B20" s="37">
@@ -18296,7 +18296,7 @@
     </row>
     <row r="21">
       <c r="A21" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*17)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B21" s="30">
@@ -18334,7 +18334,7 @@
     </row>
     <row r="22">
       <c r="A22" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*16)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B22" s="37">
@@ -18372,7 +18372,7 @@
     </row>
     <row r="23">
       <c r="A23" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*15)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B23" s="30">
@@ -18410,7 +18410,7 @@
     </row>
     <row r="24">
       <c r="A24" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*14)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B24" s="37">
@@ -18448,7 +18448,7 @@
     </row>
     <row r="25">
       <c r="A25" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*13)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B25" s="30">
@@ -18486,7 +18486,7 @@
     </row>
     <row r="26">
       <c r="A26" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*12)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B26" s="37">
@@ -18524,7 +18524,7 @@
     </row>
     <row r="27">
       <c r="A27" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*11)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B27" s="30">
@@ -18562,7 +18562,7 @@
     </row>
     <row r="28">
       <c r="A28" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*10)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B28" s="37">
@@ -18600,7 +18600,7 @@
     </row>
     <row r="29">
       <c r="A29" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*9)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B29" s="30">
@@ -18638,7 +18638,7 @@
     </row>
     <row r="30">
       <c r="A30" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*8)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B30" s="37">
@@ -18676,7 +18676,7 @@
     </row>
     <row r="31">
       <c r="A31" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*7)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B31" s="30">
@@ -18714,7 +18714,7 @@
     </row>
     <row r="32">
       <c r="A32" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*6)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B32" s="37">
@@ -18752,7 +18752,7 @@
     </row>
     <row r="33">
       <c r="A33" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*5)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B33" s="30">
@@ -18790,7 +18790,7 @@
     </row>
     <row r="34">
       <c r="A34" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*4)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B34" s="37">
@@ -18828,7 +18828,7 @@
     </row>
     <row r="35">
       <c r="A35" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*3)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B35" s="30">
@@ -18866,7 +18866,7 @@
     </row>
     <row r="36">
       <c r="A36" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*2)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B36" s="37">
@@ -18904,7 +18904,7 @@
     </row>
     <row r="37">
       <c r="A37" s="29">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*1)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B37" s="30">
@@ -18942,7 +18942,7 @@
     </row>
     <row r="38">
       <c r="A38" s="36">
-        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM")</f>
+        <f>TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0),"DD.MM")&amp;"–"&amp;TEXT((($E$3-WEEKDAY($E$3,2)+1-7*(WEEKDAY($E$3,2)&lt;7))-7*0)+6,"DD.MM.YYYY")</f>
         <v/>
       </c>
       <c r="B38" s="37">
@@ -19073,7 +19073,7 @@
     </row>
     <row r="43">
       <c r="A43" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-11))</f>
         <v/>
       </c>
       <c r="B43" s="30">
@@ -19111,7 +19111,7 @@
     </row>
     <row r="44">
       <c r="A44" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-10))</f>
         <v/>
       </c>
       <c r="B44" s="37">
@@ -19149,7 +19149,7 @@
     </row>
     <row r="45">
       <c r="A45" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-9))</f>
         <v/>
       </c>
       <c r="B45" s="30">
@@ -19187,7 +19187,7 @@
     </row>
     <row r="46">
       <c r="A46" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-8))</f>
         <v/>
       </c>
       <c r="B46" s="37">
@@ -19225,7 +19225,7 @@
     </row>
     <row r="47">
       <c r="A47" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-7))</f>
         <v/>
       </c>
       <c r="B47" s="30">
@@ -19263,7 +19263,7 @@
     </row>
     <row r="48">
       <c r="A48" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-6))</f>
         <v/>
       </c>
       <c r="B48" s="37">
@@ -19301,7 +19301,7 @@
     </row>
     <row r="49">
       <c r="A49" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-5))</f>
         <v/>
       </c>
       <c r="B49" s="30">
@@ -19339,7 +19339,7 @@
     </row>
     <row r="50">
       <c r="A50" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-4))</f>
         <v/>
       </c>
       <c r="B50" s="37">
@@ -19377,7 +19377,7 @@
     </row>
     <row r="51">
       <c r="A51" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-3))</f>
         <v/>
       </c>
       <c r="B51" s="30">
@@ -19415,7 +19415,7 @@
     </row>
     <row r="52">
       <c r="A52" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-2))</f>
         <v/>
       </c>
       <c r="B52" s="37">
@@ -19453,7 +19453,7 @@
     </row>
     <row r="53">
       <c r="A53" s="29">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),-1))</f>
         <v/>
       </c>
       <c r="B53" s="30">
@@ -19491,7 +19491,7 @@
     </row>
     <row r="54">
       <c r="A54" s="36">
-        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")</f>
+        <f>CHOOSE(MONTH(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0)),"Январь","Февраль","Март","Апрель","Май","Июнь","Июль","Август","Сентябрь","Октябрь","Ноябрь","Декабрь")&amp;" "&amp;YEAR(EDATE(EDATE(DATE(YEAR($E$3),MONTH($E$3),1),-($E$3&lt;EOMONTH($E$3,0))),0))</f>
         <v/>
       </c>
       <c r="B54" s="37">

</xml_diff>

<commit_message>
Update once a day at 01:00 Moscow time with data up to yesterday
The trigger now runs daily at 01:00 in Europe/Moscow, set on the trigger
itself so the project's timezone doesn't matter, and loads days up to
yesterday (on 28.10 at 01:00 — up to 27.10). The report's end date is
yesterday, the last full day. Partial rows for today left by the
3-hour version are dropped on the next load.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kPBSYq9ZY5XtdXkATthy6
</commit_message>
<xml_diff>
--- a/sova-report/sova-report.xlsx
+++ b/sova-report/sova-report.xlsx
@@ -2898,7 +2898,7 @@
     </row>
     <row r="4">
       <c r="H4" s="11">
-        <f>IF(AND(ISNUMBER(H3),H3&gt;$E$3),"⚠ Дата «с» позже сегодняшней",IF(ISNUMBER(H3),"Сравнение — с предыдущим периодом той же длины. Очистите поле, чтобы считать с 1-го числа месяца.","«С» — вручную (двойной щелчок — календарь), пусто — с 1-го числа месяца. «По» — всегда сегодня."))</f>
+        <f>IF(AND(ISNUMBER(H3),H3&gt;$E$3),"⚠ Дата «с» позже вчерашней",IF(ISNUMBER(H3),"Сравнение — с предыдущим периодом той же длины. Очистите поле, чтобы считать с 1-го числа месяца.","«С» — вручную (двойной щелчок — календарь), пусто — с 1-го числа месяца. «По» — всегда вчера."))</f>
         <v/>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
     </row>
     <row r="4">
       <c r="H4" s="11">
-        <f>IF(AND(ISNUMBER(H3),H3&gt;$E$3),"⚠ Дата «с» позже сегодняшней",IF(ISNUMBER(H3),"Сравнение — с предыдущим периодом той же длины. Очистите поле, чтобы считать с 1-го числа месяца.","«С» — вручную (двойной щелчок — календарь), пусто — с 1-го числа месяца. «По» — всегда сегодня."))</f>
+        <f>IF(AND(ISNUMBER(H3),H3&gt;$E$3),"⚠ Дата «с» позже вчерашней",IF(ISNUMBER(H3),"Сравнение — с предыдущим периодом той же длины. Очистите поле, чтобы считать с 1-го числа месяца.","«С» — вручную (двойной щелчок — календарь), пусто — с 1-го числа месяца. «По» — всегда вчера."))</f>
         <v/>
       </c>
     </row>
@@ -12716,7 +12716,7 @@
     </row>
     <row r="4">
       <c r="H4" s="11">
-        <f>IF(AND(ISNUMBER(H3),H3&gt;$E$3),"⚠ Дата «с» позже сегодняшней",IF(ISNUMBER(H3),"Сравнение — с предыдущим периодом той же длины. Очистите поле, чтобы считать с 1-го числа месяца.","«С» — вручную (двойной щелчок — календарь), пусто — с 1-го числа месяца. «По» — всегда сегодня."))</f>
+        <f>IF(AND(ISNUMBER(H3),H3&gt;$E$3),"⚠ Дата «с» позже вчерашней",IF(ISNUMBER(H3),"Сравнение — с предыдущим периодом той же длины. Очистите поле, чтобы считать с 1-го числа месяца.","«С» — вручную (двойной щелчок — календарь), пусто — с 1-го числа месяца. «По» — всегда вчера."))</f>
         <v/>
       </c>
     </row>
@@ -18913,7 +18913,7 @@
     </row>
     <row r="4">
       <c r="H4" s="11">
-        <f>IF(AND(ISNUMBER(H3),H3&gt;$E$3),"⚠ Дата «с» позже сегодняшней",IF(ISNUMBER(H3),"Сравнение — с предыдущим периодом той же длины. Очистите поле, чтобы считать с 1-го числа месяца.","«С» — вручную (двойной щелчок — календарь), пусто — с 1-го числа месяца. «По» — всегда сегодня."))</f>
+        <f>IF(AND(ISNUMBER(H3),H3&gt;$E$3),"⚠ Дата «с» позже вчерашней",IF(ISNUMBER(H3),"Сравнение — с предыдущим периодом той же длины. Очистите поле, чтобы считать с 1-го числа месяца.","«С» — вручную (двойной щелчок — календарь), пусто — с 1-го числа месяца. «По» — всегда вчера."))</f>
         <v/>
       </c>
     </row>
@@ -25051,12 +25051,12 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>TODAY()</f>
+        <f>TODAY()-1</f>
         <v/>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>← всегда сегодня</t>
+          <t>← всегда вчера (последний полный день)</t>
         </is>
       </c>
     </row>

</xml_diff>